<commit_message>
Workflow: ExcelConvertTableToHtml, Activity: Multiple Assign - strStyleValue & Content, updated, to change width from % to px. Config value: ColNo_Width, added, to set report desired columns width in px.
</commit_message>
<xml_diff>
--- a/Data/Config_Process_Name_Dispatcher.xlsx
+++ b/Data/Config_Process_Name_Dispatcher.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PiotrDane\02 Firma\02 Nowy Kontrahent\03 PGajewski\My Templates\WindowsC_Dispatcher_Template\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5728DA47-D566-4C84-9DFF-AFE19C4638C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3778EF-E269-4E23-8EB0-08B463833DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="81">
   <si>
     <t>Name</t>
   </si>
@@ -373,6 +373,27 @@
 &lt;/html&gt;</t>
   </si>
   <si>
+    <t>{"TO":{"Min":2, "VShort":4, "Short":8, "Medium":16, "Long":64, "VLong":256, "Max":512},
+"TOms":{"Min":2000, "VShort":4000, "Short":8000, "Medium":16000, "Long":64000, "VLong":256000, "Max":512000},
+"DEL":{"D1":1, "D2":2, "D3":3, "D4":4, "D6":6},
+"RS":{"ShowRobotStatus":{"NR":2, "TS":5}, "FoldersFilesCreateDelete":{"NR":3, "TS":4}, "AppXYLogin":{"NR":2, "TS":6}, "ExcelGetTable":{"NR":2, "TS":6}, "OrchestratorGetSetActivities":{"NR":2, "TS":5}, "OutlookGetEmails":{"NR":2, "TS":8}, "OutlookSendEmail":{"NR":2, "TS":6}, "APIRunQuery":{"NR":2, "TS":6}, "SQLRunQuery":{"NR":2, "TS":6}},
+"SE":["SE00: Critical error while initializing the environment."], 
+"AE":["AE00: Unexpected application exception.", 
+"AE01: Robot couldn't login to AppXY.", 
+"AE02: Robot couldn't logout from AppXY."], 
+"BE":["BE00: Missing input data: {0}, aborting process."],
+"Status": ["Added to queue.", "Skipped, already exists in queue."]}</t>
+  </si>
+  <si>
+    <t>ColNo_Width</t>
+  </si>
+  <si>
+    <t>Dictionary where key is report column number, value is corresponding desired width in px.</t>
+  </si>
+  <si>
+    <t>{1:150, 2:350}</t>
+  </si>
+  <si>
     <t>&lt;!DOCTYPE html&gt;
 &lt;html&gt;
 &lt;head&gt;
@@ -383,7 +404,7 @@
   background-color: white;
 }
 #tableMain {
-  width: 450px;
+  width: 500px;
   margin-top: 30px;
   margin-left: 20px;
   background-color: #EDEDED;
@@ -461,18 +482,6 @@
 &lt;/body&gt;
 &lt;/html&gt;</t>
   </si>
-  <si>
-    <t>{"TO":{"Min":2, "VShort":4, "Short":8, "Medium":16, "Long":64, "VLong":256, "Max":512},
-"TOms":{"Min":2000, "VShort":4000, "Short":8000, "Medium":16000, "Long":64000, "VLong":256000, "Max":512000},
-"DEL":{"D1":1, "D2":2, "D3":3, "D4":4, "D6":6},
-"RS":{"ShowRobotStatus":{"NR":2, "TS":5}, "FoldersFilesCreateDelete":{"NR":3, "TS":4}, "AppXYLogin":{"NR":2, "TS":6}, "ExcelGetTable":{"NR":2, "TS":6}, "OrchestratorGetSetActivities":{"NR":2, "TS":5}, "OutlookGetEmails":{"NR":2, "TS":8}, "OutlookSendEmail":{"NR":2, "TS":6}, "APIRunQuery":{"NR":2, "TS":6}, "SQLRunQuery":{"NR":2, "TS":6}},
-"SE":["SE00: Critical error while initializing the environment."], 
-"AE":["AE00: Unexpected application exception.", 
-"AE01: Robot couldn't login to AppXY.", 
-"AE02: Robot couldn't logout from AppXY."], 
-"BE":["BE00: Missing input data: {0}, aborting process."],
-"Status": ["Added to queue.", "Skipped, already exists in queue."]}</t>
-  </si>
 </sst>
 </file>
 
@@ -529,12 +538,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -849,7 +859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z24"/>
+  <dimension ref="A1:Z25"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="2" width="50.77734375" customWidth="1"/>
@@ -929,7 +939,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -1016,76 +1026,87 @@
       <c r="A16" t="s">
         <v>49</v>
       </c>
-      <c r="B16" t="s">
-        <v>76</v>
+      <c r="B16" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="C16" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" t="s">
-        <v>58</v>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" t="s">
-        <v>53</v>
+        <v>47</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
         <v>51</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>75</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C21" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
         <v>45</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>64</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C25" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Workflow: GetTransactionData, updated. Workflow: QueuePopulate, updated. Config file updated.
</commit_message>
<xml_diff>
--- a/Data/Config_Process_Name_Dispatcher.xlsx
+++ b/Data/Config_Process_Name_Dispatcher.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PiotrDane\02 Firma\02 Nowy Kontrahent\03 PGajewski\My Templates\WindowsC_Dispatcher_Template\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3778EF-E269-4E23-8EB0-08B463833DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD43B79A-86EF-45FF-B130-011A42C8DC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -263,6 +263,28 @@
     <t>ExcelInputSheet, Process_Name_InputFileSheet</t>
   </si>
   <si>
+    <t>ColNo_Width</t>
+  </si>
+  <si>
+    <t>Dictionary where key is report column number, value is corresponding desired width in px.</t>
+  </si>
+  <si>
+    <t>{1:150, 2:350}</t>
+  </si>
+  <si>
+    <t>{"TO":{"Min":2, "VShort":4, "Short":8, "Medium":16, "Long":64, "VLong":256, "Max":512},
+"TOms":{"Min":2000, "VShort":4000, "Short":8000, "Medium":16000, "Long":64000, "VLong":256000, "Max":512000},
+"DEL":{"D1":1, "D2":2, "D3":3, "D4":4, "D6":6},
+"RS":{"ShowRobotStatus":{"NR":2, "TS":5}, "FoldersFilesCreateDelete":{"NR":3, "TS":4}, "AppXYLogin":{"NR":2, "TS":6}, "ExcelGetTable":{"NR":2, "TS":6}, "OrchestratorGetSetActivities":{"NR":2, "TS":5}, "OutlookGetEmails":{"NR":2, "TS":8}, "OutlookSendEmail":{"NR":2, "TS":6}, "APIRunQuery":{"NR":2, "TS":6}, "SQLRunQuery":{"NR":2, "TS":6}},
+"SE":["SE00: Critical error while initializing the environment."], 
+"AE":["AE00: Unexpected application exception.", 
+"AE01: Robot couldn't login to AppXY.", 
+"AE02: Robot couldn't logout from AppXY."], 
+"BE":["BE00: Missing input data: {0}, aborting process.", 
+"BE01: Invalid date provided in row: {0}, column: {1}."],
+"Status": ["Added to queue.", "Skipped, already exists in queue."]}</t>
+  </si>
+  <si>
     <t>&lt;!DOCTYPE html&gt;
 &lt;html&gt;
 &lt;head&gt;
@@ -276,7 +298,6 @@
   padding: 12px;
 }
 #tableMain {
-  width: 90%;
   max-width: 600px;
   margin-top: 30px;
   margin-left: 20px;
@@ -373,27 +394,6 @@
 &lt;/html&gt;</t>
   </si>
   <si>
-    <t>{"TO":{"Min":2, "VShort":4, "Short":8, "Medium":16, "Long":64, "VLong":256, "Max":512},
-"TOms":{"Min":2000, "VShort":4000, "Short":8000, "Medium":16000, "Long":64000, "VLong":256000, "Max":512000},
-"DEL":{"D1":1, "D2":2, "D3":3, "D4":4, "D6":6},
-"RS":{"ShowRobotStatus":{"NR":2, "TS":5}, "FoldersFilesCreateDelete":{"NR":3, "TS":4}, "AppXYLogin":{"NR":2, "TS":6}, "ExcelGetTable":{"NR":2, "TS":6}, "OrchestratorGetSetActivities":{"NR":2, "TS":5}, "OutlookGetEmails":{"NR":2, "TS":8}, "OutlookSendEmail":{"NR":2, "TS":6}, "APIRunQuery":{"NR":2, "TS":6}, "SQLRunQuery":{"NR":2, "TS":6}},
-"SE":["SE00: Critical error while initializing the environment."], 
-"AE":["AE00: Unexpected application exception.", 
-"AE01: Robot couldn't login to AppXY.", 
-"AE02: Robot couldn't logout from AppXY."], 
-"BE":["BE00: Missing input data: {0}, aborting process."],
-"Status": ["Added to queue.", "Skipped, already exists in queue."]}</t>
-  </si>
-  <si>
-    <t>ColNo_Width</t>
-  </si>
-  <si>
-    <t>Dictionary where key is report column number, value is corresponding desired width in px.</t>
-  </si>
-  <si>
-    <t>{1:150, 2:350}</t>
-  </si>
-  <si>
     <t>&lt;!DOCTYPE html&gt;
 &lt;html&gt;
 &lt;head&gt;
@@ -415,7 +415,7 @@
   white-space: normal;
 }
 #tableMainHeader {
-  background-color: #27CCF5;
+  background-color: #2ecc71;
   padding: 14px;
   font-size: 16px;
   font-weight: bold;
@@ -939,7 +939,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -1035,13 +1035,13 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" t="s">
         <v>77</v>
       </c>
-      <c r="B17" t="s">
-        <v>79</v>
-      </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1071,7 +1071,7 @@
         <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C21" t="s">
         <v>57</v>

</xml_diff>